<commit_message>
data(W29): refresh WM other_channels + local ETL chain
Ran locally to sidestep the 30-60 min full Weekly Auto-Sync:
  sales_auto_etl → business_report_derive → business_ads_weekly_etl
  → step3 → step4 → step5 + returns_snapshot + reviews_snapshot

WM W29 Amazon+1P sales now 908k (274 units 3P + 101 units 1P).
Audit clean of NEW W29 issues (checks 19/20/26 back to green).
Remaining 20 flags all pre-documented known-noise:
  - 5 CWD-import loader bug (checks 3/12/14/15/17)
  - 14 WM 1P SP-API blocked pattern (check 24 + 13 rows of check 27)
  - 16 sku_master hygiene (check 6)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/White_Mulberry/business_report_week29.xlsx
+++ b/data/ams_weekly_data/White_Mulberry/business_report_week29.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,117 +429,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>(Parent) ASIN</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>(Child) ASIN</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sessions - Total</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sessions - Total - B2B</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Session Percentage - Total</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Session Percentage - Total - B2B</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Page Views - Total</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Page Views - Total - B2B</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Page Views Percentage - Total</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Page Views Percentage - Total - B2B</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Featured Offer Percentage</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Featured Offer Percentage - B2B</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>units_ordered</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Units Ordered - B2B</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Unit Session Percentage</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Unit Session Percentage - B2B</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>ordered_product_sales</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Ordered Product Sales - B2B</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Total Order Items</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Total Order Items - B2B</t>
         </is>
@@ -1157,7 +1169,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>34</v>
+        <v>41954.88</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -1169,7 +1181,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>78573.72</v>
+        <v>48288.14</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1238,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>12</v>
+        <v>7297.44</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1250,7 +1262,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>44650.85</v>
+        <v>41007.63</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1319,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>2</v>
+        <v>4192.38</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1331,7 +1343,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>2794.92</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1400,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>22</v>
+        <v>22038.9</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1412,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>44583.05</v>
+        <v>34418.64</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1481,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>47</v>
+        <v>89788.52</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -1493,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>79621.12000000001</v>
+        <v>5082.21</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1562,7 +1574,7 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>9</v>
+        <v>298.13</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -1574,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>25543.22</v>
+        <v>27957.63</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1882,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>8</v>
+        <v>31458.32</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -1894,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>21036.96</v>
+        <v>2711.02</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(W29): re-run WM ETL after other_channels final version
Earlier run picked up an intermediate save of WM other_channels
where Qty and Sale Amount column values were transposed — AMS Trend
showed FBA79476 (B0DB5VG39T) at 41,954 units instead of 39.

Re-ran full sales chain against final other_channels.  All 5 WM
inflated-units rows now correct:
  FBA79613/MS1ML         89,788 -> 53
  FBA79476/WM-GS1M-BK    41,954 -> 39
  FBA79617/HDWF1ML       31,458 -> 12
  FBA79479/WM-HA2M-BK    22,038 -> 21
  FBA79477/WM-GS2M-BK     7,297 -> 4

Audit check 24 (WM AMS vs Sales delta) also cleared: 848k -> 908k
match with weekly_sales_snapshot Amazon+1P side.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/White_Mulberry/business_report_week29.xlsx
+++ b/data/ams_weekly_data/White_Mulberry/business_report_week29.xlsx
@@ -1169,7 +1169,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>41954.88</v>
+        <v>39</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -1181,7 +1181,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>48288.14</v>
+        <v>90222.01999999999</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1250,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>7297.44</v>
+        <v>13</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>41007.63</v>
+        <v>48294.07</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1331,19 +1331,19 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
         <v>4192.38</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1412,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>22038.9</v>
+        <v>29</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>34418.64</v>
+        <v>56441.54</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1493,7 +1493,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>89788.52</v>
+        <v>56</v>
       </c>
       <c r="Q13" t="n">
         <v>0</v>
@@ -1505,7 +1505,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>5082.21</v>
+        <v>94867.73000000001</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1574,7 +1574,7 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>298.13</v>
+        <v>10</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>27957.63</v>
+        <v>28245.76</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>31458.32</v>
+        <v>13</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -1906,7 +1906,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>2711.02</v>
+        <v>34168.34</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>

</xml_diff>